<commit_message>
Add Invoice no. as the first column in the expense import template
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/TEMPLATE_รายจ่าย.xlsx
+++ b/public/templates/TEMPLATE_รายจ่าย.xlsx
@@ -397,19 +397,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="28.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="28.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
     <col min="10" max="10" width="14.83203125" customWidth="1"/>
     <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -429,182 +430,197 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>Invoice no.</v>
+      </c>
+      <c r="B4" t="str">
         <v>วันที่สั่งสินค้า ★</v>
       </c>
-      <c r="B4" t="str">
+      <c r="C4" t="str">
         <v>หมวดหมู่สินค้า ★</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>รายละเอียด ★</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>รหัสไซท์งาน ★</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>ชื่อ Supplier ★</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>VAT/NO VAT ★</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>มูลค่าก่อน VAT (บาท) ★</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>มูลค่ารวม VAT (บาท) ★</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>วิธีชำระ ★</v>
       </c>
-      <c r="J4" t="str">
+      <c r="K4" t="str">
         <v>วันที่ชำระ</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>สถานะจ่าย</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>TEXT</v>
+      </c>
+      <c r="B5" t="str">
         <v>DATE</v>
       </c>
-      <c r="B5" t="str">
+      <c r="C5" t="str">
         <v>เลือกหมวด</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>TEXT</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>FX-XXXX-XXX</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>TEXT (สร้างใหม่อัตโนมัติถ้าไม่พบ)</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>VAT/NO VAT</v>
-      </c>
-      <c r="G5" t="str">
-        <v>NUMBER</v>
       </c>
       <c r="H5" t="str">
         <v>NUMBER</v>
       </c>
       <c r="I5" t="str">
+        <v>NUMBER</v>
+      </c>
+      <c r="J5" t="str">
         <v>CASH/CREDIT/TRANSFER/CHECK</v>
       </c>
-      <c r="J5" t="str">
+      <c r="K5" t="str">
         <v>DATE</v>
       </c>
-      <c r="K5" t="str">
+      <c r="L5" t="str">
         <v>paid/pending/...</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>INV-6603/BT001</v>
+      </c>
+      <c r="B6" t="str">
         <v>2026-06-01</v>
       </c>
-      <c r="B6" t="str">
+      <c r="C6" t="str">
         <v>ค่าอลูมิเนียม/เหล็ก</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>อลูมิเนียมโปรไฟล์ 6m</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>FX-2026-016</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>บ.แม่น้ำมิทอล ซัพพลาย จำกัด</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>VAT</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>79439.25</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>85000</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>CREDIT</v>
       </c>
-      <c r="J6" t="str">
+      <c r="K6" t="str">
         <v>2026-07-01</v>
       </c>
-      <c r="K6" t="str">
+      <c r="L6" t="str">
         <v>pending</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>IV6802052</v>
+      </c>
+      <c r="B7" t="str">
         <v>2026-06-03</v>
       </c>
-      <c r="B7" t="str">
+      <c r="C7" t="str">
         <v>ค่ากระจก</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>กระจกเทมเปอร์ 12mm</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>FX-2026-013</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>บ.ช.เจริญกลาส จำกัด</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>VAT</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>112149.53</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>120000</v>
       </c>
-      <c r="I7" t="str">
+      <c r="J7" t="str">
         <v>TRANSFER</v>
       </c>
-      <c r="J7" t="str">
+      <c r="K7" t="str">
         <v>2026-06-03</v>
       </c>
-      <c r="K7" t="str">
+      <c r="L7" t="str">
         <v>paid</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
         <v>2026-06-20</v>
       </c>
-      <c r="B8" t="str">
+      <c r="C8" t="str">
         <v>ค่าอุปกรณ์</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>น็อต สกรู อุปกรณ์รวม</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>FX-2026-013</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>บ.พีพีวาย โปรดักส์ จำกัด</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>NO VAT</v>
-      </c>
-      <c r="G8">
-        <v>3200</v>
       </c>
       <c r="H8">
         <v>3200</v>
       </c>
-      <c r="I8" t="str">
+      <c r="I8">
+        <v>3200</v>
+      </c>
+      <c r="J8" t="str">
         <v>CASH</v>
       </c>
-      <c r="J8" t="str">
+      <c r="K8" t="str">
         <v>2026-06-20</v>
       </c>
-      <c r="K8" t="str">
+      <c r="L8" t="str">
         <v>paid</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>